<commit_message>
updates with word pair diffs
</commit_message>
<xml_diff>
--- a/Aim2/Aim2_Data/aim2_timestamps_final_2.xlsx
+++ b/Aim2/Aim2_Data/aim2_timestamps_final_2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/krg/Documents/Rise_new/Aim2/Aim2_Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/krg/Documents/RISE_7_12/Aim2/Aim2_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C5D64C1-4B33-AD45-8AB4-6FF00FCD0179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E55C8DC-F673-1E46-B96E-144A508C7F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="580" yWindow="1440" windowWidth="28220" windowHeight="16180" activeTab="5" xr2:uid="{1905D5AD-B59A-4349-BC54-AD7B07C29ACC}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1412" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="289">
   <si>
     <t>Frame Start</t>
   </si>
@@ -904,6 +904,12 @@
   </si>
   <si>
     <t xml:space="preserve"> Frame End</t>
+  </si>
+  <si>
+    <t>sentence_onset_frame</t>
+  </si>
+  <si>
+    <t>target_word_onset_frame</t>
   </si>
 </sst>
 </file>
@@ -5545,15 +5551,17 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{745B2EC6-FBC4-384D-8EF7-4158DEE7776E}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -5569,8 +5577,14 @@
       <c r="E1" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F1" t="s">
+        <v>287</v>
+      </c>
+      <c r="G1" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5581,13 +5595,20 @@
         <v>60</v>
       </c>
       <c r="D2">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="E2" s="1">
         <v>310</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F2">
+        <v>208</v>
+      </c>
+      <c r="G2">
+        <v>228</v>
+      </c>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -5598,13 +5619,20 @@
         <v>62</v>
       </c>
       <c r="D3">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="E3" s="1">
         <v>520</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F3">
+        <v>418</v>
+      </c>
+      <c r="G3">
+        <v>437</v>
+      </c>
+      <c r="H3" s="1"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5615,13 +5643,20 @@
         <v>64</v>
       </c>
       <c r="D4">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="E4" s="1">
         <v>730</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F4">
+        <v>635</v>
+      </c>
+      <c r="G4">
+        <v>664</v>
+      </c>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -5632,13 +5667,20 @@
         <v>66</v>
       </c>
       <c r="D5">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="E5" s="1">
         <v>940</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F5">
+        <v>835</v>
+      </c>
+      <c r="G5">
+        <v>853</v>
+      </c>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -5649,13 +5691,20 @@
         <v>68</v>
       </c>
       <c r="D6">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="E6" s="1">
         <v>1150</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6">
+        <v>1049</v>
+      </c>
+      <c r="G6">
+        <v>1067</v>
+      </c>
+      <c r="H6" s="1"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -5666,13 +5715,20 @@
         <v>71</v>
       </c>
       <c r="D7">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="E7" s="1">
-        <v>1360</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+        <v>1361</v>
+      </c>
+      <c r="F7">
+        <v>1258</v>
+      </c>
+      <c r="G7">
+        <v>1274</v>
+      </c>
+      <c r="H7" s="1"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -5683,13 +5739,20 @@
         <v>72</v>
       </c>
       <c r="D8">
-        <v>1423</v>
+        <v>1421</v>
       </c>
       <c r="E8" s="1">
-        <v>1570</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+        <v>1571</v>
+      </c>
+      <c r="F8">
+        <v>1466</v>
+      </c>
+      <c r="G8">
+        <v>1495</v>
+      </c>
+      <c r="H8" s="1"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -5700,13 +5763,20 @@
         <v>73</v>
       </c>
       <c r="D9">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="E9" s="1">
-        <v>1780</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+        <v>1781</v>
+      </c>
+      <c r="F9">
+        <v>1679</v>
+      </c>
+      <c r="G9">
+        <v>1703</v>
+      </c>
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -5717,13 +5787,20 @@
         <v>74</v>
       </c>
       <c r="D10">
-        <v>1843</v>
+        <v>1841</v>
       </c>
       <c r="E10" s="1">
-        <v>1990</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+        <v>1991</v>
+      </c>
+      <c r="F10">
+        <v>1885</v>
+      </c>
+      <c r="G10">
+        <v>1903</v>
+      </c>
+      <c r="H10" s="1"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -5734,13 +5811,20 @@
         <v>75</v>
       </c>
       <c r="D11">
-        <v>2052</v>
+        <v>2051</v>
       </c>
       <c r="E11" s="1">
         <v>2201</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F11">
+        <v>2099</v>
+      </c>
+      <c r="G11">
+        <v>2118</v>
+      </c>
+      <c r="H11" s="1"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
         <f>A11+1</f>
         <v>11</v>
@@ -5752,13 +5836,20 @@
         <v>60</v>
       </c>
       <c r="D12">
-        <v>2263</v>
+        <v>2262</v>
       </c>
       <c r="E12" s="1">
         <v>2412</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F12">
+        <v>2308</v>
+      </c>
+      <c r="G12">
+        <v>2328</v>
+      </c>
+      <c r="H12" s="1"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <f t="shared" ref="A13:A21" si="0">A12+1</f>
         <v>12</v>
@@ -5770,13 +5861,20 @@
         <v>62</v>
       </c>
       <c r="D13">
-        <v>2474</v>
+        <v>2472</v>
       </c>
       <c r="E13" s="1">
         <v>2622</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13">
+        <v>2518</v>
+      </c>
+      <c r="G13">
+        <v>2537</v>
+      </c>
+      <c r="H13" s="1"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -5788,13 +5886,20 @@
         <v>66</v>
       </c>
       <c r="D14">
-        <v>2684</v>
+        <v>2682</v>
       </c>
       <c r="E14" s="1">
         <v>2832</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14">
+        <v>2730</v>
+      </c>
+      <c r="G14">
+        <v>2748</v>
+      </c>
+      <c r="H14" s="1"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -5806,13 +5911,20 @@
         <v>64</v>
       </c>
       <c r="D15">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="E15" s="1">
         <v>3042</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F15">
+        <v>2944</v>
+      </c>
+      <c r="G15">
+        <v>2973</v>
+      </c>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -5824,13 +5936,20 @@
         <v>68</v>
       </c>
       <c r="D16">
-        <v>3103</v>
+        <v>3102</v>
       </c>
       <c r="E16" s="1">
         <v>3252</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F16">
+        <v>3150</v>
+      </c>
+      <c r="G16">
+        <v>3167</v>
+      </c>
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -5842,13 +5961,20 @@
         <v>73</v>
       </c>
       <c r="D17">
-        <v>3314</v>
+        <v>3311</v>
       </c>
       <c r="E17" s="1">
-        <v>3460</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+        <v>3461</v>
+      </c>
+      <c r="F17">
+        <v>3358</v>
+      </c>
+      <c r="G17">
+        <v>3383</v>
+      </c>
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -5860,13 +5986,20 @@
         <v>71</v>
       </c>
       <c r="D18">
-        <v>3522</v>
+        <v>3521</v>
       </c>
       <c r="E18" s="1">
-        <v>3670</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+        <v>3671</v>
+      </c>
+      <c r="F18">
+        <v>3565</v>
+      </c>
+      <c r="G18">
+        <v>3584</v>
+      </c>
+      <c r="H18" s="1"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -5878,13 +6011,20 @@
         <v>72</v>
       </c>
       <c r="D19">
-        <v>3735</v>
+        <v>3731</v>
       </c>
       <c r="E19" s="1">
-        <v>3880</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+        <v>3881</v>
+      </c>
+      <c r="F19">
+        <v>3775</v>
+      </c>
+      <c r="G19">
+        <v>3806</v>
+      </c>
+      <c r="H19" s="1"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -5896,13 +6036,20 @@
         <v>74</v>
       </c>
       <c r="D20">
-        <v>3945</v>
+        <v>3941</v>
       </c>
       <c r="E20" s="1">
-        <v>4090</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+        <v>4091</v>
+      </c>
+      <c r="F20">
+        <v>3981</v>
+      </c>
+      <c r="G20">
+        <v>4001</v>
+      </c>
+      <c r="H20" s="1"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -5914,11 +6061,18 @@
         <v>75</v>
       </c>
       <c r="D21">
-        <v>4154</v>
+        <v>4151</v>
       </c>
       <c r="E21" s="1">
-        <v>4300</v>
-      </c>
+        <v>4301</v>
+      </c>
+      <c r="F21">
+        <v>4197</v>
+      </c>
+      <c r="G21">
+        <v>4218</v>
+      </c>
+      <c r="H21" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9570,15 +9724,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="6c0d6bb4-bf93-46e5-af3e-76fbe0d2898f">
@@ -9587,6 +9732,15 @@
     <TaxCatchAll xmlns="897aa84e-6803-47c8-b68c-17d5fde4eba2" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9856,14 +10010,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0CDED83-EA4E-4F36-A05F-0665C2CE98F5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6730D68A-F459-44B9-B55A-08A4C6EDF8D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -9877,6 +10023,14 @@
     <ds:schemaRef ds:uri="897aa84e-6803-47c8-b68c-17d5fde4eba2"/>
     <ds:schemaRef ds:uri="cb5fc986-ca15-48a6-9872-3e00e06f3290"/>
     <ds:schemaRef ds:uri="6c0d6bb4-bf93-46e5-af3e-76fbe0d2898f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0CDED83-EA4E-4F36-A05F-0665C2CE98F5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>